<commit_message>
Filtre cible TPE/PME (<100 salariés) joignable + module taille
- equiprospect/taille.py : classe chaque prospect par taille d'entreprise estimée
  et accessibilité (écarte grands groupes >100 et célébrités/grandes fortunes)
- commande `python -m equiprospect pme` : marque taille_estimee/cible_accessible
  et exporte data/prospects_pme.csv (88 cibles TPE/PME joignables sur 228)
- +8 dirigeants de TPE/PME cavaliers sourcés (LinkedIn X-ray small-company)
- Excel régénérés : prospects.xlsx + prospects_pme.xlsx

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSYywU174tb3YwVqt48yV7
</commit_message>
<xml_diff>
--- a/data/prospects.xlsx
+++ b/data/prospects.xlsx
@@ -422,26 +422,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q221"/>
+  <dimension ref="A1:S229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -530,6 +532,16 @@
           <t>score</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>taille_estimee</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>cible_accessible</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -613,6 +625,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -696,6 +718,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -775,6 +807,16 @@
           <t>49.0</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -854,6 +896,16 @@
           <t>49.0</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -937,6 +989,16 @@
           <t>88.2</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1020,6 +1082,16 @@
           <t>72.0</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1103,6 +1175,16 @@
           <t>85.5</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1182,6 +1264,16 @@
           <t>68.8</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1265,6 +1357,16 @@
           <t>68.8</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1348,6 +1450,16 @@
           <t>53.5</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1431,6 +1543,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1514,6 +1636,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1597,6 +1729,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1680,6 +1822,16 @@
           <t>61.2</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1763,6 +1915,16 @@
           <t>52.5</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1846,6 +2008,16 @@
           <t>81.0</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1929,6 +2101,16 @@
           <t>81.0</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2012,6 +2194,16 @@
           <t>88.2</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2095,6 +2287,16 @@
           <t>85.5</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2178,6 +2380,16 @@
           <t>38.0</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2261,6 +2473,16 @@
           <t>81.0</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2344,6 +2566,16 @@
           <t>65.0</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2427,6 +2659,16 @@
           <t>65.0</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2506,6 +2748,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2589,6 +2841,16 @@
           <t>42.5</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2672,6 +2934,16 @@
           <t>72.0</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2755,6 +3027,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2838,6 +3120,16 @@
           <t>72.7</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2921,6 +3213,16 @@
           <t>68.8</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3004,6 +3306,16 @@
           <t>65.0</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3087,6 +3399,16 @@
           <t>68.0</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3170,6 +3492,16 @@
           <t>61.2</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3253,6 +3585,16 @@
           <t>36.7</t>
         </is>
       </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3336,6 +3678,16 @@
           <t>47.2</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3419,6 +3771,16 @@
           <t>47.2</t>
         </is>
       </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3502,6 +3864,16 @@
           <t>47.2</t>
         </is>
       </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3585,6 +3957,16 @@
           <t>47.2</t>
         </is>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3668,6 +4050,16 @@
           <t>36.7</t>
         </is>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3747,6 +4139,16 @@
           <t>36.7</t>
         </is>
       </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3830,6 +4232,16 @@
           <t>50.4</t>
         </is>
       </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3913,6 +4325,16 @@
           <t>50.4</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3996,6 +4418,16 @@
           <t>47.2</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4075,6 +4507,16 @@
           <t>44.1</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4154,6 +4596,16 @@
           <t>29.4</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4237,6 +4689,16 @@
           <t>68.8</t>
         </is>
       </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4318,6 +4780,16 @@
       <c r="Q47" t="inlineStr">
         <is>
           <t>50.4</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -4395,6 +4867,16 @@
           <t>70.0</t>
         </is>
       </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4474,6 +4956,16 @@
           <t>31.8</t>
         </is>
       </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4553,6 +5045,16 @@
           <t>63.0</t>
         </is>
       </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4632,6 +5134,16 @@
           <t>16.8</t>
         </is>
       </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4715,6 +5227,16 @@
           <t>14.7</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4794,6 +5316,16 @@
           <t>12.2</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4873,6 +5405,16 @@
           <t>12.2</t>
         </is>
       </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4956,6 +5498,16 @@
           <t>42.0</t>
         </is>
       </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5039,6 +5591,16 @@
           <t>42.0</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5118,6 +5680,16 @@
           <t>63.0</t>
         </is>
       </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5195,6 +5767,16 @@
       <c r="Q58" t="inlineStr">
         <is>
           <t>42.0</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -5272,6 +5854,16 @@
           <t>70.0</t>
         </is>
       </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5349,6 +5941,16 @@
       <c r="Q60" t="inlineStr">
         <is>
           <t>31.5</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -5426,6 +6028,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5501,6 +6113,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5576,6 +6198,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5653,6 +6285,16 @@
       <c r="Q64" t="inlineStr">
         <is>
           <t>28.0</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -5730,6 +6372,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5805,6 +6457,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5880,6 +6542,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5959,6 +6631,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6032,6 +6714,16 @@
       <c r="Q69" t="inlineStr">
         <is>
           <t>0.0</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -6105,6 +6797,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6176,6 +6878,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6251,6 +6963,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6330,6 +7052,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6405,6 +7137,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6482,6 +7224,16 @@
       <c r="Q75" t="inlineStr">
         <is>
           <t>31.5</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -6555,6 +7307,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6634,6 +7396,16 @@
           <t>28.4</t>
         </is>
       </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6717,6 +7489,16 @@
           <t>42.0</t>
         </is>
       </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6796,6 +7578,16 @@
           <t>63.0</t>
         </is>
       </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6875,6 +7667,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6954,6 +7756,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7033,6 +7845,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7116,6 +7938,16 @@
           <t>42.0</t>
         </is>
       </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7193,6 +8025,16 @@
       <c r="Q84" t="inlineStr">
         <is>
           <t>42.0</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -7270,6 +8112,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7347,6 +8199,16 @@
       <c r="Q86" t="inlineStr">
         <is>
           <t>14.7</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
     </row>
@@ -7420,6 +8282,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7499,6 +8371,16 @@
           <t>34.7</t>
         </is>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7578,6 +8460,16 @@
           <t>63.0</t>
         </is>
       </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7661,6 +8553,16 @@
           <t>25.2</t>
         </is>
       </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7744,6 +8646,16 @@
           <t>22.0</t>
         </is>
       </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7827,6 +8739,16 @@
           <t>31.5</t>
         </is>
       </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7910,6 +8832,16 @@
           <t>28.0</t>
         </is>
       </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7987,6 +8919,16 @@
       <c r="Q94" t="inlineStr">
         <is>
           <t>0.0</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -8064,6 +9006,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8147,6 +9099,16 @@
           <t>63.0</t>
         </is>
       </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8226,6 +9188,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8305,6 +9277,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8384,6 +9366,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8467,6 +9459,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8550,6 +9552,16 @@
           <t>81.0</t>
         </is>
       </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8633,6 +9645,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8716,6 +9738,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8795,6 +9827,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8878,6 +9920,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8961,6 +10013,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -9040,6 +10102,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9119,6 +10191,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9198,6 +10280,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9277,6 +10369,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9356,6 +10458,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9435,6 +10547,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9512,6 +10634,16 @@
       <c r="Q113" t="inlineStr">
         <is>
           <t>0.0</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
         </is>
       </c>
     </row>
@@ -9589,6 +10721,16 @@
           <t>18.9</t>
         </is>
       </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9668,6 +10810,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -9743,6 +10895,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -9822,6 +10984,16 @@
           <t>14.7</t>
         </is>
       </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -9901,6 +11073,16 @@
           <t>14.7</t>
         </is>
       </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -9980,6 +11162,16 @@
           <t>12.2</t>
         </is>
       </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -10055,6 +11247,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -10130,6 +11332,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -10203,6 +11415,16 @@
       <c r="Q122" t="inlineStr">
         <is>
           <t>0.0</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -10276,6 +11498,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -10355,6 +11587,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -10434,6 +11676,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -10513,6 +11765,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -10592,6 +11854,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -10671,6 +11943,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -10750,6 +12032,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -10829,6 +12121,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -10908,6 +12210,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -10987,6 +12299,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -11066,6 +12388,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -11145,6 +12477,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -11224,6 +12566,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -11303,6 +12655,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -11382,6 +12744,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -11461,6 +12833,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -11540,6 +12922,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -11619,6 +13011,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -11698,6 +13100,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -11773,6 +13185,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -11848,6 +13270,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -11923,6 +13355,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -11998,6 +13440,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -12073,6 +13525,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -12148,6 +13610,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -12227,6 +13699,16 @@
           <t>17.5</t>
         </is>
       </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -12306,6 +13788,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -12385,6 +13877,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -12464,6 +13966,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -12541,6 +14053,16 @@
       <c r="Q152" t="inlineStr">
         <is>
           <t>49.7</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
@@ -12614,6 +14136,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -12689,6 +14221,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -12764,6 +14306,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -12839,6 +14391,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>grande entreprise (&gt;100)</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -12914,6 +14476,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -12993,6 +14565,16 @@
           <t>38.2</t>
         </is>
       </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>grande fortune / célébrité</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -13072,6 +14654,16 @@
           <t>35.0</t>
         </is>
       </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -13151,6 +14743,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -13230,6 +14832,16 @@
           <t>25.2</t>
         </is>
       </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -13309,6 +14921,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -13388,6 +15010,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -13467,6 +15099,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -13546,6 +15188,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -13625,6 +15277,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -13704,6 +15366,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -13783,6 +15455,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -13862,6 +15544,16 @@
           <t>63.0</t>
         </is>
       </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -13941,6 +15633,16 @@
           <t>35.0</t>
         </is>
       </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -14020,6 +15722,16 @@
           <t>49.0</t>
         </is>
       </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -14099,6 +15811,16 @@
           <t>49.0</t>
         </is>
       </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -14178,6 +15900,16 @@
           <t>49.0</t>
         </is>
       </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -14257,6 +15989,16 @@
           <t>49.0</t>
         </is>
       </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -14336,6 +16078,16 @@
           <t>49.0</t>
         </is>
       </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -14411,6 +16163,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -14486,6 +16248,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -14561,6 +16333,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -14636,6 +16418,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -14711,6 +16503,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -14786,6 +16588,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -14861,6 +16673,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -14940,6 +16762,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -15019,6 +16851,16 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -15098,6 +16940,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S185" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -15177,6 +17029,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -15260,6 +17122,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -15339,6 +17211,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -15418,6 +17300,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -15497,6 +17389,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -15576,6 +17478,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S191" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -15655,6 +17567,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -15734,6 +17656,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S193" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -15813,6 +17745,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -15892,6 +17834,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -15971,6 +17923,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S196" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -16050,6 +18012,16 @@
           <t>27.6</t>
         </is>
       </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -16129,6 +18101,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -16208,6 +18190,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -16287,6 +18279,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -16366,6 +18368,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -16445,6 +18457,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -16524,6 +18546,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -16603,6 +18635,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -16682,6 +18724,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S205" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -16761,6 +18813,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S206" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -16840,6 +18902,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S207" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -16919,6 +18991,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S208" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -16998,6 +19080,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -17077,6 +19169,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -17156,6 +19258,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -17235,6 +19347,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S212" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -17314,6 +19436,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -17393,6 +19525,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -17472,6 +19614,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -17551,6 +19703,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -17630,6 +19792,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -17709,6 +19881,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -17788,6 +19970,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -17867,6 +20059,16 @@
           <t>49.7</t>
         </is>
       </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>association/fédération (bénévole)</t>
+        </is>
+      </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>a_confirmer</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -17944,6 +20146,696 @@
       <c r="Q221" t="inlineStr">
         <is>
           <t>49.7</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Gérald Brault</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Dirigeant (distributeur de produits équins)</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Distribution équine (TPE)</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/g%C3%A9rald-brault-07161a97</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr"/>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Cavalier pratiquant affiché sur le profil (dirigeant de TPE)</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>Profil « Cavalier, distributeur de produits equins » — cavalier pratiquant (NB: déjà dans la filière équine)</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/g%C3%A9rald-brault-07161a97</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr"/>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Lamia Moraine</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Cofondatrice &amp; Directrice Générale</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Inovelite</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/lamia-moraine-inovelite</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr"/>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>Profil remonté sur requête « cavalière » + cofondatrice/DG (PME)</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/lamia-moraine-inovelite</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr"/>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Isabelle Delannoy</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Présidente</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>L'Entreprise Symbiotique</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/isabelle-delannoy-8337225</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr"/>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Profil remonté sur requête « cavalière » + présidente (petite structure)</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/isabelle-delannoy-8337225</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr"/>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Eve Pauvert</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Dirigeante</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Facilis.fr (TPE/PME, Alsace)</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/eve-pauvert-dirigeante-facilis-cse-tpe-pme-alsace-grandest</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Profil remonté sur requête « dirigeante » TPE/PME + « cavalière »/concours</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/eve-pauvert-dirigeante-facilis-cse-tpe-pme-alsace-grandest</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr"/>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Vanessa Logerais</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Fondatrice / dirigeante</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Parangone (agence)</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr"/>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/vanessa-logerais-parangone</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr"/>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Profil remonté sur requête « dirigeante » PME + « cavalière »</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/vanessa-logerais-parangone</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr"/>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Rafaëlle Rivier</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Présidente</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>MOMA Consulting</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr"/>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/rafaelle-rivier</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr"/>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>Profil remonté sur requête « dirigeante » + « cavalière »/concours (conseil, PME)</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/rafaelle-rivier</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr"/>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Pauline Laigneau</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Fondatrice</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Gemmyo / Demian Education</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr"/>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/pauline-laigneau</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr"/>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Profil remonté sur requête « cavalière » + fondatrice (à confirmer; taille Gemmyo à vérifier)</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/pauline-laigneau</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O228" t="inlineStr"/>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Caroline Clavel</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Gérante</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Écurie (TPE)</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr"/>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/caroline-clavel-40ba79197</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr"/>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Cavalière pratiquante affichée sur le profil (gérante de TPE)</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>Profil « Gérante - Cavalière » — cavalière pratiquante (NB: gère une écurie, filière équine)</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/caroline-clavel-40ba79197</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>aucun</t>
+        </is>
+      </c>
+      <c r="O229" t="inlineStr"/>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
+3 dirigeants de PME cavaliers (231 au total; 91 cibles TPE/PME joignables)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSYywU174tb3YwVqt48yV7
</commit_message>
<xml_diff>
--- a/data/prospects.xlsx
+++ b/data/prospects.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S229"/>
+  <dimension ref="A1:S232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20839,6 +20839,273 @@
         </is>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Marie Dauxerre</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Gérante fondatrice</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Abeille Informatique (PME)</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr"/>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/marie-dauxerre-4298b858</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Profil « gérante fondatrice » remonté sur requête équitation/cheval + PME</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/marie-dauxerre-4298b858</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>incertain</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>affinite_cheval</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>mention équestre générique</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Joëlle Daumas-Guirado</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>CEO (créatrice de crampons pneus)</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>UGIGRIP (PME industrielle)</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/jo%C3%ABlle-daumas-guirado/en</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>Profil CEO PME remonté sur requête « cavalier/équitation » + indépendant</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/jo%C3%ABlle-daumas-guirado/en</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>incertain</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>affinite_cheval</t>
+        </is>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>mention équestre générique</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>B-profil LinkedIn à qualifier</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Samuel Usureau</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Directeur Commercial</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>JDA Dijon</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/samuel-usureau-88b293139</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr"/>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Indice équestre détecté via requête Google croisée (à confirmer sur le profil)</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>Profil remonté sur requête « directeur » + dressage/saut d'obstacles amateur</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/in/samuel-usureau-88b293139</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>cavalier_pratiquant</t>
+        </is>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>dressage</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>49.0</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>TPE/PME estimée (&lt;100)</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>